<commit_message>
Add clinical QA results and update model benchmarking paths
- Introduced new clinical QA results in JSON format for various queries related to COPD and diabetes.
- Updated paths in `generate_plots.py` and `run_models.py` to reflect new directory structure for results and metrics.
- Added new metrics CSV for clinical results and RAGChecker outputs for improved analysis and benchmarking.
</commit_message>
<xml_diff>
--- a/model_benchmarking/results/factual/results_full/metrics.xlsx
+++ b/model_benchmarking/results/factual/results_full/metrics.xlsx
@@ -5960,7 +5960,7 @@
         </is>
       </c>
       <c r="C185" t="n">
-        <v>2440.4608</v>
+        <v>18.049</v>
       </c>
       <c r="D185" t="n">
         <v>2312</v>
@@ -5972,7 +5972,7 @@
         <v>1552</v>
       </c>
       <c r="G185" t="n">
-        <v>0.74</v>
+        <v>100.28</v>
       </c>
       <c r="H185" t="n">
         <v>0.06586</v>
@@ -5990,7 +5990,7 @@
         </is>
       </c>
       <c r="C186" t="n">
-        <v>2425.8588</v>
+        <v>18.049</v>
       </c>
       <c r="D186" t="n">
         <v>752</v>
@@ -6002,7 +6002,7 @@
         <v>2588</v>
       </c>
       <c r="G186" t="n">
-        <v>1.13</v>
+        <v>151.81</v>
       </c>
       <c r="H186" t="n">
         <v>0.08595999999999999</v>
@@ -6080,7 +6080,7 @@
         </is>
       </c>
       <c r="C189" t="n">
-        <v>2455.1266</v>
+        <v>18.049</v>
       </c>
       <c r="D189" t="n">
         <v>636</v>
@@ -6092,7 +6092,7 @@
         <v>516</v>
       </c>
       <c r="G189" t="n">
-        <v>0.28</v>
+        <v>37.95</v>
       </c>
       <c r="H189" t="n">
         <v>0.02373</v>
@@ -6110,7 +6110,7 @@
         </is>
       </c>
       <c r="C190" t="n">
-        <v>2418.2932</v>
+        <v>18.049</v>
       </c>
       <c r="D190" t="n">
         <v>744</v>
@@ -6122,7 +6122,7 @@
         <v>516</v>
       </c>
       <c r="G190" t="n">
-        <v>0.32</v>
+        <v>42.99</v>
       </c>
       <c r="H190" t="n">
         <v>0.027</v>
@@ -6170,7 +6170,7 @@
         </is>
       </c>
       <c r="C192" t="n">
-        <v>2542.9004</v>
+        <v>18.049</v>
       </c>
       <c r="D192" t="n">
         <v>102</v>
@@ -6182,7 +6182,7 @@
         <v>2070</v>
       </c>
       <c r="G192" t="n">
-        <v>0.83</v>
+        <v>117.24</v>
       </c>
       <c r="H192" t="n">
         <v>0.06399000000000001</v>
@@ -11180,7 +11180,7 @@
         </is>
       </c>
       <c r="C359" t="n">
-        <v>2083.6092</v>
+        <v>18.3993</v>
       </c>
       <c r="D359" t="n">
         <v>1225</v>
@@ -11192,7 +11192,7 @@
         <v>1034</v>
       </c>
       <c r="G359" t="n">
-        <v>0.54</v>
+        <v>61.31</v>
       </c>
       <c r="H359" t="n">
         <v>0.01998</v>
@@ -11210,7 +11210,7 @@
         </is>
       </c>
       <c r="C360" t="n">
-        <v>2107.9185</v>
+        <v>18.3993</v>
       </c>
       <c r="D360" t="n">
         <v>1747</v>
@@ -11222,7 +11222,7 @@
         <v>2588</v>
       </c>
       <c r="G360" t="n">
-        <v>1.35</v>
+        <v>154.46</v>
       </c>
       <c r="H360" t="n">
         <v>0.047</v>
@@ -11240,7 +11240,7 @@
         </is>
       </c>
       <c r="C361" t="n">
-        <v>2135.2969</v>
+        <v>18.3993</v>
       </c>
       <c r="D361" t="n">
         <v>1999</v>
@@ -11252,7 +11252,7 @@
         <v>4734</v>
       </c>
       <c r="G361" t="n">
-        <v>2.55</v>
+        <v>295.83</v>
       </c>
       <c r="H361" t="n">
         <v>0.08663999999999999</v>
@@ -11450,7 +11450,7 @@
         </is>
       </c>
       <c r="C368" t="n">
-        <v>2108.387</v>
+        <v>18.3993</v>
       </c>
       <c r="D368" t="n">
         <v>102</v>
@@ -11462,7 +11462,7 @@
         <v>1552</v>
       </c>
       <c r="G368" t="n">
-        <v>0.75</v>
+        <v>86.31</v>
       </c>
       <c r="H368" t="n">
         <v>0.02407</v>
@@ -11540,7 +11540,7 @@
         </is>
       </c>
       <c r="C371" t="n">
-        <v>2130.8456</v>
+        <v>18.3993</v>
       </c>
       <c r="D371" t="n">
         <v>9015</v>
@@ -11552,7 +11552,7 @@
         <v>1552</v>
       </c>
       <c r="G371" t="n">
-        <v>0.87</v>
+        <v>101.25</v>
       </c>
       <c r="H371" t="n">
         <v>0.05048</v>

</xml_diff>